<commit_message>
Termincado el Sprint_2, Terminado Requisitos funcionales del codigo, a Revision de los no funcionales
</commit_message>
<xml_diff>
--- a/Avance.xlsx
+++ b/Avance.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\universidad\6_Semestre\Ing_Software_2\banco-preguntas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{081C995F-38FA-4E94-BBE8-E3380D6A9338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B5B948D-9B5C-40F7-BF36-7EB7F2A7E470}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11700" yWindow="825" windowWidth="17325" windowHeight="11295" xr2:uid="{A4552BDB-F8A7-4E28-A504-476D727EEB1E}"/>
   </bookViews>
@@ -1614,6 +1614,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2312625-4BC1-4C6F-AD18-BB88F450FCD7}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="B2:D19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1821,7 +1824,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup scale="83" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
   <tableParts count="1">
     <tablePart r:id="rId3"/>

</xml_diff>